<commit_message>
Update DB schema, add UI mockup, revise docs
Update FirestoreSchema.xlsx to reflect schema changes, add Designs/UI-Frontend/PaperDesign.JPEG as a new UI mockup, and apply revisions to Documentation/LSEP.docx and Documentation/report.docx. These changes align the database design, UI concept, and documentation with recent feature and UX updates.
</commit_message>
<xml_diff>
--- a/Designs/DatabaseDesign/FirestoreSchema.xlsx
+++ b/Designs/DatabaseDesign/FirestoreSchema.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matthew\Github\Year3\COMP3000-Computing-Project\Designs\DatabaseDesign\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mattr\Github\Matt-Fish-COMP3000-Computing-Project\Designs\DatabaseDesign\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F40DEBD-29C8-4C2B-8675-85A8120A4DD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19E9EFA2-7BC4-424A-A6B4-7705E14C155F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="39495" yWindow="2880" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Schema" sheetId="1" r:id="rId1"/>
+    <sheet name="Final Schema" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="89">
   <si>
     <t>Users</t>
   </si>
@@ -120,12 +121,246 @@
 assigned_to: user_uid // Optional
 </t>
   </si>
+  <si>
+    <t>Field Name</t>
+  </si>
+  <si>
+    <t>Data Type</t>
+  </si>
+  <si>
+    <t>Security / Notes</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>String</t>
+  </si>
+  <si>
+    <t>Plaintext - User's display name</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>Plaintext - Google OAuth email</t>
+  </si>
+  <si>
+    <t>role</t>
+  </si>
+  <si>
+    <t>Plaintext - e.g., 'admin', 'analyst' (RBAC)</t>
+  </si>
+  <si>
+    <t>tech_level</t>
+  </si>
+  <si>
+    <t>Determines Gemini API persona prompt</t>
+  </si>
+  <si>
+    <t>notification_level</t>
+  </si>
+  <si>
+    <t>Threshold for email alerts (e.g., 'critical')</t>
+  </si>
+  <si>
+    <t>app_notification_level</t>
+  </si>
+  <si>
+    <t>Threshold for in-app UI alerts</t>
+  </si>
+  <si>
+    <t>cleared_notifications</t>
+  </si>
+  <si>
+    <t>Array</t>
+  </si>
+  <si>
+    <t>Tracks which alerts the user has dismissed</t>
+  </si>
+  <si>
+    <t>created_at</t>
+  </si>
+  <si>
+    <t>Timestamp</t>
+  </si>
+  <si>
+    <t>Server-side account creation time</t>
+  </si>
+  <si>
+    <t>USERS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collection: </t>
+  </si>
+  <si>
+    <t>Manages identity, Role-Based Access Control (RBAC), and user configuration.</t>
+  </si>
+  <si>
+    <t>Firebase Auth UID</t>
+  </si>
+  <si>
+    <t>incidents</t>
+  </si>
+  <si>
+    <t>The central repository for processed network threats and AI analysis.</t>
+  </si>
+  <si>
+    <t>Auto-generated Firestore UID</t>
+  </si>
+  <si>
+    <t>is_encrypted</t>
+  </si>
+  <si>
+    <t>Boolean</t>
+  </si>
+  <si>
+    <t>Flag to trigger frontend decryption logic</t>
+  </si>
+  <si>
+    <t>data</t>
+  </si>
+  <si>
+    <t>String (Ciphertext)</t>
+  </si>
+  <si>
+    <r>
+      <t>[AES Encrypted]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> The raw sanitised log data</t>
+    </r>
+  </si>
+  <si>
+    <t>ai_insights</t>
+  </si>
+  <si>
+    <t>Array (Ciphertext)</t>
+  </si>
+  <si>
+    <r>
+      <t>[AES Encrypted]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> The LLM summary and mitigation steps</t>
+    </r>
+  </si>
+  <si>
+    <t>user_notes</t>
+  </si>
+  <si>
+    <r>
+      <t>[AES Encrypted]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Manual notes added by analysts</t>
+    </r>
+  </si>
+  <si>
+    <t>risk_score</t>
+  </si>
+  <si>
+    <t>Integer</t>
+  </si>
+  <si>
+    <t>Plaintext (1-10) - Used for quick Dashboard UI sorting</t>
+  </si>
+  <si>
+    <t>analysis_status</t>
+  </si>
+  <si>
+    <t>Plaintext - e.g., 'AI_Analysis_Complete', 'resolved'</t>
+  </si>
+  <si>
+    <t>assigned_to</t>
+  </si>
+  <si>
+    <t>Plaintext - User UID of the assigned analyst</t>
+  </si>
+  <si>
+    <t>completed_steps</t>
+  </si>
+  <si>
+    <t>Array [Integers]</t>
+  </si>
+  <si>
+    <t>Plaintext - Tracks mitigation progress checkboxes</t>
+  </si>
+  <si>
+    <t>timestamp</t>
+  </si>
+  <si>
+    <t>Server-side time of log ingestion</t>
+  </si>
+  <si>
+    <t>An immutable forensic ledger tracking all API interactions.</t>
+  </si>
+  <si>
+    <t>client_ip</t>
+  </si>
+  <si>
+    <t>The IP address making the HTTP request</t>
+  </si>
+  <si>
+    <t>method</t>
+  </si>
+  <si>
+    <t>e.g., 'GET', 'POST', 'PATCH'</t>
+  </si>
+  <si>
+    <t>path</t>
+  </si>
+  <si>
+    <t>The specific FastAPI endpoint accessed</t>
+  </si>
+  <si>
+    <t>status_code</t>
+  </si>
+  <si>
+    <t>e.g., 200 (Success), 403 (Forbidden)</t>
+  </si>
+  <si>
+    <t>process_time</t>
+  </si>
+  <si>
+    <t>Float</t>
+  </si>
+  <si>
+    <t>Server execution time (for performance monitoring)</t>
+  </si>
+  <si>
+    <t>user_agent</t>
+  </si>
+  <si>
+    <t>Browser/Client software identification</t>
+  </si>
+  <si>
+    <t>Server-side execution time</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -141,6 +376,25 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Google Sans Text"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -150,7 +404,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -173,11 +427,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -190,6 +459,25 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -471,15 +759,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:F10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="13.109375" customWidth="1"/>
-    <col min="3" max="3" width="70.21875" customWidth="1"/>
-    <col min="5" max="5" width="11.88671875" customWidth="1"/>
-    <col min="6" max="6" width="55.88671875" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" customWidth="1"/>
+    <col min="3" max="3" width="70.28515625" customWidth="1"/>
+    <col min="5" max="5" width="11.85546875" customWidth="1"/>
+    <col min="6" max="6" width="55.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:6">
       <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
@@ -493,7 +781,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="2:6" ht="31.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:6" ht="31.9" customHeight="1">
       <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
@@ -507,7 +795,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:6">
       <c r="B4" s="2" t="s">
         <v>4</v>
       </c>
@@ -521,7 +809,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="2:6" ht="119.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:6" ht="119.45" customHeight="1">
       <c r="B5" s="2" t="s">
         <v>6</v>
       </c>
@@ -535,7 +823,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:6">
       <c r="B7" s="1" t="s">
         <v>1</v>
       </c>
@@ -549,7 +837,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:6">
       <c r="B8" s="2" t="s">
         <v>9</v>
       </c>
@@ -563,7 +851,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:6">
       <c r="B9" s="2" t="s">
         <v>11</v>
       </c>
@@ -577,7 +865,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="2:6" ht="189" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:6" ht="204" customHeight="1">
       <c r="B10" s="2" t="s">
         <v>13</v>
       </c>
@@ -594,4 +882,374 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFF608B7-1954-44BC-A72A-023492BACE65}">
+  <dimension ref="B2:H28"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="19.85546875" customWidth="1"/>
+    <col min="3" max="3" width="36.5703125" customWidth="1"/>
+    <col min="4" max="4" width="42.42578125" customWidth="1"/>
+    <col min="5" max="5" width="37.140625" customWidth="1"/>
+    <col min="6" max="6" width="20.85546875" customWidth="1"/>
+    <col min="7" max="7" width="33.85546875" customWidth="1"/>
+    <col min="8" max="8" width="54.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:8">
+      <c r="D2" s="9"/>
+    </row>
+    <row r="3" spans="2:8" ht="25.5" customHeight="1">
+      <c r="B3" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="G3" s="12" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8" ht="35.25" customHeight="1">
+      <c r="B4" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" ht="22.5" customHeight="1">
+      <c r="B5" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" ht="22.5" customHeight="1" thickBot="1"/>
+    <row r="7" spans="2:8" ht="26.25" customHeight="1" thickBot="1">
+      <c r="B7" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" ht="26.25" customHeight="1" thickBot="1">
+      <c r="B8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" ht="26.25" customHeight="1" thickBot="1">
+      <c r="B9" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" ht="26.25" customHeight="1" thickBot="1">
+      <c r="B10" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="11" spans="2:8" ht="26.25" customHeight="1" thickBot="1">
+      <c r="B11" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8" ht="26.25" customHeight="1" thickBot="1">
+      <c r="B12" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" ht="26.25" customHeight="1" thickBot="1">
+      <c r="B13" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="H13" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8" ht="26.25" customHeight="1" thickBot="1">
+      <c r="B14" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="H14" s="8" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8" ht="26.25" customHeight="1" thickBot="1">
+      <c r="B15" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="H15" s="8" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="16" spans="2:8" ht="12.75" customHeight="1" thickBot="1">
+      <c r="F16" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="H16" s="8" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4">
+      <c r="B17" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" ht="30">
+      <c r="B18" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4">
+      <c r="B19" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4" ht="15.75" thickBot="1"/>
+    <row r="21" spans="2:4" ht="26.25" customHeight="1" thickBot="1">
+      <c r="B21" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4" ht="26.25" customHeight="1" thickBot="1">
+      <c r="B22" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4" ht="26.25" customHeight="1" thickBot="1">
+      <c r="B23" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="24" spans="2:4" ht="26.25" customHeight="1" thickBot="1">
+      <c r="B24" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="25" spans="2:4" ht="26.25" customHeight="1" thickBot="1">
+      <c r="B25" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="26" spans="2:4" ht="26.25" customHeight="1" thickBot="1">
+      <c r="B26" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="D26" s="8" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="27" spans="2:4" ht="26.25" customHeight="1" thickBot="1">
+      <c r="B27" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="28" spans="2:4" ht="26.25" customHeight="1" thickBot="1">
+      <c r="B28" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>